<commit_message>
fix(reconstruction): refine p10 model audit evidence
</commit_message>
<xml_diff>
--- a/_pipelines/02_task_datasets/reconstruction/_outputs/p10_model_results/track_model_metrics.xlsx
+++ b/_pipelines/02_task_datasets/reconstruction/_outputs/p10_model_results/track_model_metrics.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="model metrics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型指标" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -645,7 +645,7 @@
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -761,7 +761,7 @@
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -877,7 +877,7 @@
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -993,7 +993,7 @@
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -1109,7 +1109,7 @@
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
@@ -1225,7 +1225,7 @@
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
@@ -1341,7 +1341,7 @@
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -1457,7 +1457,7 @@
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
@@ -1573,7 +1573,7 @@
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
@@ -1689,7 +1689,7 @@
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
@@ -1805,7 +1805,7 @@
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
@@ -1921,7 +1921,7 @@
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
@@ -2037,7 +2037,7 @@
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
@@ -2153,7 +2153,7 @@
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
@@ -2269,7 +2269,7 @@
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
@@ -2385,7 +2385,7 @@
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
@@ -2501,7 +2501,7 @@
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
@@ -2617,7 +2617,7 @@
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
@@ -2733,7 +2733,7 @@
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
@@ -2849,7 +2849,7 @@
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
@@ -2965,7 +2965,7 @@
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
@@ -3081,7 +3081,7 @@
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
@@ -3197,7 +3197,7 @@
       <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
@@ -3313,7 +3313,7 @@
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
@@ -3429,7 +3429,7 @@
       <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
@@ -3545,7 +3545,7 @@
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
@@ -3661,7 +3661,7 @@
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
@@ -3777,7 +3777,7 @@
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
@@ -3893,7 +3893,7 @@
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
@@ -4009,7 +4009,7 @@
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
@@ -4125,7 +4125,7 @@
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
@@ -4241,7 +4241,7 @@
       <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
@@ -4357,7 +4357,7 @@
       <c r="V34" t="inlineStr"/>
       <c r="W34" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
@@ -4473,7 +4473,7 @@
       <c r="V35" t="inlineStr"/>
       <c r="W35" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
@@ -4589,7 +4589,7 @@
       <c r="V36" t="inlineStr"/>
       <c r="W36" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
@@ -4705,7 +4705,7 @@
       <c r="V37" t="inlineStr"/>
       <c r="W37" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
@@ -4821,7 +4821,7 @@
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
@@ -4937,7 +4937,7 @@
       <c r="V39" t="inlineStr"/>
       <c r="W39" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X39" t="inlineStr">
@@ -5053,12 +5053,12 @@
       <c r="V40" t="inlineStr"/>
       <c r="W40" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>pretraining improves the same adapter over random init, but the same split/sample universe still sits far above the PyKrige baseline</t>
+          <t>foundation gain is real versus random init, but end-to-end performance remains non_beneficial against PyKrige on the same strict sample universe; audited checkpoints include PATCH_SHAPE=(9,20,18), grid_shape_kji=[63,100,108], coordinate roundtrip max abs error=0.0, and mode-specific mask exclusion is already encoded in the archived summaries</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
@@ -5068,7 +5068,7 @@
       </c>
       <c r="Z40" t="inlineStr">
         <is>
-          <t>frozen_test_accessed=False; same_validation_sample_universe=True</t>
+          <t>frozen_test_accessed=False; same_validation_sample_universe=True; adapter_decoder_output_shape_not_exposed_in_archived_summary</t>
         </is>
       </c>
     </row>
@@ -5169,12 +5169,12 @@
       <c r="V41" t="inlineStr"/>
       <c r="W41" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>same architecture without pretraining has far higher error on the same strict fold universe</t>
+          <t>same architecture without pretraining has far higher error on the same strict fold universe; this confirms the foundation gain but not promotion</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
@@ -5184,7 +5184,7 @@
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>comparison is same-arch random initialization against the PyKrige reference</t>
+          <t>comparison is same-arch random initialization against the PyKrige reference; same split/sample universe as pretrained run</t>
         </is>
       </c>
     </row>
@@ -5285,12 +5285,12 @@
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>PyKrige is the strongest reference on the same strict sample universe</t>
+          <t>PyKrige is the strongest reference on the same strict sample universe; serves as the end-to-end baseline that OpenMind does not beat</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>strong_baseline_macro_fold_rmse comes from the same fold universe as the foundation comparison</t>
+          <t>strong_baseline_macro_fold_rmse comes from the same fold universe as the foundation comparison; no frozen holdout was used here</t>
         </is>
       </c>
     </row>
@@ -5401,7 +5401,7 @@
       <c r="V43" t="inlineStr"/>
       <c r="W43" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X43" t="inlineStr">
@@ -5517,7 +5517,7 @@
       <c r="V44" t="inlineStr"/>
       <c r="W44" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X44" t="inlineStr">
@@ -5633,7 +5633,7 @@
       <c r="V45" t="inlineStr"/>
       <c r="W45" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X45" t="inlineStr">
@@ -5749,7 +5749,7 @@
       <c r="V46" t="inlineStr"/>
       <c r="W46" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X46" t="inlineStr">
@@ -5865,7 +5865,7 @@
       <c r="V47" t="inlineStr"/>
       <c r="W47" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X47" t="inlineStr">
@@ -5981,7 +5981,7 @@
       <c r="V48" t="inlineStr"/>
       <c r="W48" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X48" t="inlineStr">
@@ -6097,7 +6097,7 @@
       <c r="V49" t="inlineStr"/>
       <c r="W49" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X49" t="inlineStr">
@@ -6213,7 +6213,7 @@
       <c r="V50" t="inlineStr"/>
       <c r="W50" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X50" t="inlineStr">
@@ -6329,7 +6329,7 @@
       <c r="V51" t="inlineStr"/>
       <c r="W51" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X51" t="inlineStr">
@@ -6445,7 +6445,7 @@
       <c r="V52" t="inlineStr"/>
       <c r="W52" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X52" t="inlineStr">
@@ -6561,7 +6561,7 @@
       <c r="V53" t="inlineStr"/>
       <c r="W53" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X53" t="inlineStr">
@@ -6677,7 +6677,7 @@
       <c r="V54" t="inlineStr"/>
       <c r="W54" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X54" t="inlineStr">
@@ -6793,7 +6793,7 @@
       <c r="V55" t="inlineStr"/>
       <c r="W55" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X55" t="inlineStr">
@@ -6909,7 +6909,7 @@
       <c r="V56" t="inlineStr"/>
       <c r="W56" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X56" t="inlineStr">
@@ -7025,7 +7025,7 @@
       <c r="V57" t="inlineStr"/>
       <c r="W57" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X57" t="inlineStr">
@@ -7145,12 +7145,12 @@
       </c>
       <c r="W58" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test</t>
+          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test; stage4_mode=strict</t>
         </is>
       </c>
       <c r="Y58" t="inlineStr">
@@ -7160,7 +7160,7 @@
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout</t>
+          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout; confirmation_only</t>
         </is>
       </c>
     </row>
@@ -7265,12 +7265,12 @@
       </c>
       <c r="W59" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test</t>
+          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test; stage4_mode=strict</t>
         </is>
       </c>
       <c r="Y59" t="inlineStr">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="Z59" t="inlineStr">
         <is>
-          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout</t>
+          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout; confirmation_only</t>
         </is>
       </c>
     </row>
@@ -7385,12 +7385,12 @@
       </c>
       <c r="W60" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test</t>
+          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test; stage4_mode=strict</t>
         </is>
       </c>
       <c r="Y60" t="inlineStr">
@@ -7400,7 +7400,7 @@
       </c>
       <c r="Z60" t="inlineStr">
         <is>
-          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout</t>
+          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout; confirmation_only</t>
         </is>
       </c>
     </row>
@@ -7505,12 +7505,12 @@
       </c>
       <c r="W61" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test</t>
+          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test; stage4_mode=strict</t>
         </is>
       </c>
       <c r="Y61" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="Z61" t="inlineStr">
         <is>
-          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout</t>
+          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout; confirmation_only</t>
         </is>
       </c>
     </row>
@@ -7625,12 +7625,12 @@
       </c>
       <c r="W62" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test</t>
+          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test; stage4_mode=conditional</t>
         </is>
       </c>
       <c r="Y62" t="inlineStr">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="Z62" t="inlineStr">
         <is>
-          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout</t>
+          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout; confirmation_only</t>
         </is>
       </c>
     </row>
@@ -7745,12 +7745,12 @@
       </c>
       <c r="W63" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test</t>
+          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test; stage4_mode=conditional</t>
         </is>
       </c>
       <c r="Y63" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="Z63" t="inlineStr">
         <is>
-          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout</t>
+          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout; confirmation_only</t>
         </is>
       </c>
     </row>
@@ -7865,12 +7865,12 @@
       </c>
       <c r="W64" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test</t>
+          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test; stage4_mode=conditional</t>
         </is>
       </c>
       <c r="Y64" t="inlineStr">
@@ -7880,7 +7880,7 @@
       </c>
       <c r="Z64" t="inlineStr">
         <is>
-          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout</t>
+          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout; confirmation_only</t>
         </is>
       </c>
     </row>
@@ -7985,12 +7985,12 @@
       </c>
       <c r="W65" t="inlineStr">
         <is>
-          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
         </is>
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test</t>
+          <t>known-holdout confirmation on previously seen holdout, not a fresh blind test; stage4_mode=conditional</t>
         </is>
       </c>
       <c r="Y65" t="inlineStr">
@@ -8000,7 +8000,7 @@
       </c>
       <c r="Z65" t="inlineStr">
         <is>
-          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout</t>
+          <t>prior_test_consumed=True; fresh_blind=False; evidence_class=previously_seen_reusable_holdout; confirmation_only</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(reconstruction): refresh p10 audit outputs
</commit_message>
<xml_diff>
--- a/_pipelines/02_task_datasets/reconstruction/_outputs/p10_model_results/track_model_metrics.xlsx
+++ b/_pipelines/02_task_datasets/reconstruction/_outputs/p10_model_results/track_model_metrics.xlsx
@@ -645,7 +645,7 @@
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -761,7 +761,7 @@
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -877,7 +877,7 @@
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -993,7 +993,7 @@
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -1109,7 +1109,7 @@
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
@@ -1225,7 +1225,7 @@
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
@@ -1341,7 +1341,7 @@
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -1457,7 +1457,7 @@
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
@@ -1573,7 +1573,7 @@
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
@@ -1689,7 +1689,7 @@
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
@@ -1805,7 +1805,7 @@
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
@@ -1921,7 +1921,7 @@
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
@@ -2037,7 +2037,7 @@
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
@@ -2153,7 +2153,7 @@
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
@@ -2269,7 +2269,7 @@
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
@@ -2385,7 +2385,7 @@
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
@@ -2501,7 +2501,7 @@
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
@@ -2617,7 +2617,7 @@
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
@@ -2733,7 +2733,7 @@
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
@@ -2849,7 +2849,7 @@
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
@@ -2965,7 +2965,7 @@
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
@@ -3081,7 +3081,7 @@
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
@@ -3197,7 +3197,7 @@
       <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
@@ -3313,7 +3313,7 @@
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
@@ -3429,7 +3429,7 @@
       <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
@@ -3545,7 +3545,7 @@
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
@@ -3661,7 +3661,7 @@
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
@@ -3777,7 +3777,7 @@
       <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
@@ -3893,7 +3893,7 @@
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
@@ -4009,7 +4009,7 @@
       <c r="V31" t="inlineStr"/>
       <c r="W31" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
@@ -4125,7 +4125,7 @@
       <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
@@ -4241,7 +4241,7 @@
       <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
@@ -4357,7 +4357,7 @@
       <c r="V34" t="inlineStr"/>
       <c r="W34" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
@@ -4473,7 +4473,7 @@
       <c r="V35" t="inlineStr"/>
       <c r="W35" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
@@ -4589,7 +4589,7 @@
       <c r="V36" t="inlineStr"/>
       <c r="W36" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
@@ -4705,7 +4705,7 @@
       <c r="V37" t="inlineStr"/>
       <c r="W37" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
@@ -4821,7 +4821,7 @@
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
@@ -4937,7 +4937,7 @@
       <c r="V39" t="inlineStr"/>
       <c r="W39" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X39" t="inlineStr">
@@ -5053,7 +5053,7 @@
       <c r="V40" t="inlineStr"/>
       <c r="W40" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X40" t="inlineStr">
@@ -5169,7 +5169,7 @@
       <c r="V41" t="inlineStr"/>
       <c r="W41" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X41" t="inlineStr">
@@ -5285,7 +5285,7 @@
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X42" t="inlineStr">
@@ -5401,7 +5401,7 @@
       <c r="V43" t="inlineStr"/>
       <c r="W43" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X43" t="inlineStr">
@@ -5517,7 +5517,7 @@
       <c r="V44" t="inlineStr"/>
       <c r="W44" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X44" t="inlineStr">
@@ -5633,7 +5633,7 @@
       <c r="V45" t="inlineStr"/>
       <c r="W45" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X45" t="inlineStr">
@@ -5749,7 +5749,7 @@
       <c r="V46" t="inlineStr"/>
       <c r="W46" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X46" t="inlineStr">
@@ -5865,7 +5865,7 @@
       <c r="V47" t="inlineStr"/>
       <c r="W47" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X47" t="inlineStr">
@@ -5981,7 +5981,7 @@
       <c r="V48" t="inlineStr"/>
       <c r="W48" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X48" t="inlineStr">
@@ -6097,7 +6097,7 @@
       <c r="V49" t="inlineStr"/>
       <c r="W49" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X49" t="inlineStr">
@@ -6213,7 +6213,7 @@
       <c r="V50" t="inlineStr"/>
       <c r="W50" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X50" t="inlineStr">
@@ -6329,7 +6329,7 @@
       <c r="V51" t="inlineStr"/>
       <c r="W51" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X51" t="inlineStr">
@@ -6445,7 +6445,7 @@
       <c r="V52" t="inlineStr"/>
       <c r="W52" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X52" t="inlineStr">
@@ -6561,7 +6561,7 @@
       <c r="V53" t="inlineStr"/>
       <c r="W53" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X53" t="inlineStr">
@@ -6677,7 +6677,7 @@
       <c r="V54" t="inlineStr"/>
       <c r="W54" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X54" t="inlineStr">
@@ -6793,7 +6793,7 @@
       <c r="V55" t="inlineStr"/>
       <c r="W55" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X55" t="inlineStr">
@@ -6909,7 +6909,7 @@
       <c r="V56" t="inlineStr"/>
       <c r="W56" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X56" t="inlineStr">
@@ -7025,7 +7025,7 @@
       <c r="V57" t="inlineStr"/>
       <c r="W57" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X57" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="W58" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X58" t="inlineStr">
@@ -7265,7 +7265,7 @@
       </c>
       <c r="W59" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X59" t="inlineStr">
@@ -7385,7 +7385,7 @@
       </c>
       <c r="W60" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X60" t="inlineStr">
@@ -7505,7 +7505,7 @@
       </c>
       <c r="W61" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X61" t="inlineStr">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="W62" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X62" t="inlineStr">
@@ -7745,7 +7745,7 @@
       </c>
       <c r="W63" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X63" t="inlineStr">
@@ -7865,7 +7865,7 @@
       </c>
       <c r="W64" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X64" t="inlineStr">
@@ -7985,7 +7985,7 @@
       </c>
       <c r="W65" t="inlineStr">
         <is>
-          <t>e08e05a8f6e4f46d3178de3fda5216def7112c07</t>
+          <t>5685933c382b698c4cc4003780d66277f24f21a3</t>
         </is>
       </c>
       <c r="X65" t="inlineStr">

</xml_diff>